<commit_message>
ManureMgmt: Updated EF for stable losses from Swedish IIR 2025
</commit_message>
<xml_diff>
--- a/data/default/ManureMgmt.xlsx
+++ b/data/default/ManureMgmt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E10BFD5-DF70-4A22-BAE4-C5B0B3E77FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCE5617-CD6F-4CE5-9E2A-5E848FF4E913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="references" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1671" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1717" uniqueCount="216">
   <si>
     <t>value</t>
   </si>
@@ -550,9 +550,6 @@
     <t>Swedish IIR 2023 Table 5-8</t>
   </si>
   <si>
-    <t>Swedish IIR 2023 Table 5-11</t>
-  </si>
-  <si>
     <t>Swedish IIR 2023 Table 5-12</t>
   </si>
   <si>
@@ -671,6 +668,21 @@
   </si>
   <si>
     <t>OBS. Fel i källtabell (står 0,25% där)</t>
+  </si>
+  <si>
+    <t>"loose housing"</t>
+  </si>
+  <si>
+    <t>Swedish IIR 2025 Table 5-11</t>
+  </si>
+  <si>
+    <t>typo in source table</t>
+  </si>
+  <si>
+    <t>typo in source table "same as liquid"</t>
+  </si>
+  <si>
+    <t>"floor system"</t>
   </si>
 </sst>
 </file>
@@ -1432,26 +1444,8 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1467,6 +1461,24 @@
     </xf>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="9"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1815,7 +1827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O322"/>
+  <dimension ref="A1:O327"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -1844,7 +1856,7 @@
         <v>28</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>110</v>
@@ -1988,7 +2000,7 @@
         <v>3</v>
       </c>
       <c r="G6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K6" t="s">
         <v>14</v>
@@ -2123,7 +2135,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K11" t="s">
         <v>14</v>
@@ -2246,7 +2258,7 @@
         <v>9</v>
       </c>
       <c r="G16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K16" t="s">
         <v>14</v>
@@ -2366,7 +2378,7 @@
         <v>8</v>
       </c>
       <c r="G21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K21" t="s">
         <v>14</v>
@@ -2411,7 +2423,7 @@
         <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G23" t="s">
         <v>16</v>
@@ -2435,7 +2447,7 @@
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G24" t="s">
         <v>17</v>
@@ -2459,7 +2471,7 @@
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G25" t="s">
         <v>18</v>
@@ -2483,10 +2495,10 @@
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G26" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K26" t="s">
         <v>14</v>
@@ -2507,7 +2519,7 @@
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G27" t="s">
         <v>166</v>
@@ -2594,7 +2606,7 @@
         <v>48</v>
       </c>
       <c r="G31" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K31" t="s">
         <v>14</v>
@@ -2699,7 +2711,7 @@
         <v>54</v>
       </c>
       <c r="G36" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K36" t="s">
         <v>14</v>
@@ -2804,7 +2816,7 @@
         <v>35</v>
       </c>
       <c r="G41" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K41" t="s">
         <v>14</v>
@@ -2846,7 +2858,7 @@
         <v>35</v>
       </c>
       <c r="E43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G43" t="s">
         <v>16</v>
@@ -2870,7 +2882,7 @@
         <v>35</v>
       </c>
       <c r="E44" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G44" t="s">
         <v>17</v>
@@ -2894,7 +2906,7 @@
         <v>35</v>
       </c>
       <c r="E45" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G45" t="s">
         <v>18</v>
@@ -2918,10 +2930,10 @@
         <v>35</v>
       </c>
       <c r="E46" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G46" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K46" t="s">
         <v>14</v>
@@ -2942,7 +2954,7 @@
         <v>35</v>
       </c>
       <c r="E47" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G47" t="s">
         <v>166</v>
@@ -3029,7 +3041,7 @@
         <v>45</v>
       </c>
       <c r="G51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K51" t="s">
         <v>14</v>
@@ -3146,7 +3158,7 @@
         <v>47</v>
       </c>
       <c r="G56" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K56" t="s">
         <v>14</v>
@@ -3188,17 +3200,17 @@
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="44" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="44" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K61" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L61" s="6">
         <v>0</v>
@@ -3221,10 +3233,10 @@
         <v>3</v>
       </c>
       <c r="G62" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K62" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L62" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A62&amp;C62&amp;E62,MMS!$P$8:$Z$8,0))</f>
@@ -3234,7 +3246,7 @@
         <v>15</v>
       </c>
       <c r="N62" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="O62" t="s">
         <v>169</v>
@@ -3251,10 +3263,10 @@
         <v>3</v>
       </c>
       <c r="G63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K63" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L63" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A63&amp;C63&amp;E63,MMS!$P$8:$Z$8,0))</f>
@@ -3272,10 +3284,10 @@
         <v>9</v>
       </c>
       <c r="G64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K64" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L64" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A64&amp;C64&amp;E64,MMS!$P$8:$Z$8,0))</f>
@@ -3293,10 +3305,10 @@
         <v>8</v>
       </c>
       <c r="G65" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K65" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L65" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A65&amp;C65&amp;E65,MMS!$P$8:$Z$8,0))</f>
@@ -3311,13 +3323,13 @@
         <v>1</v>
       </c>
       <c r="E66" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G66" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K66" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L66" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A66&amp;C66&amp;E66,MMS!$P$8:$Z$8,0))</f>
@@ -3332,10 +3344,10 @@
         <v>48</v>
       </c>
       <c r="G67" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K67" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L67" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A67&amp;C67&amp;E67,MMS!$P$8:$Z$8,0))</f>
@@ -3350,10 +3362,10 @@
         <v>54</v>
       </c>
       <c r="G68" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K68" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L68" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A68&amp;C68&amp;E68,MMS!$P$8:$Z$8,0))</f>
@@ -3368,10 +3380,10 @@
         <v>35</v>
       </c>
       <c r="G69" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K69" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L69" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A69&amp;C69&amp;E69,MMS!$P$8:$Z$8,0))</f>
@@ -3386,13 +3398,13 @@
         <v>35</v>
       </c>
       <c r="E70" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G70" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K70" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L70" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A70&amp;C70&amp;E70,MMS!$P$8:$Z$8,0))</f>
@@ -3407,10 +3419,10 @@
         <v>45</v>
       </c>
       <c r="G71" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K71" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L71" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A71&amp;C71&amp;E71,MMS!$P$8:$Z$8,0))</f>
@@ -3428,10 +3440,10 @@
         <v>47</v>
       </c>
       <c r="G72" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K72" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L72" s="37">
         <f>INDEX(MMS!$P$16:$Z$16,MATCH(A72&amp;C72&amp;E72,MMS!$P$8:$Z$8,0))</f>
@@ -3589,7 +3601,7 @@
         <v>1</v>
       </c>
       <c r="E84" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J84" t="s">
         <v>121</v>
@@ -4133,7 +4145,7 @@
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G120" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K120" t="s">
         <v>56</v>
@@ -4165,7 +4177,7 @@
         <v>57</v>
       </c>
       <c r="N121" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="O121" t="s">
         <v>66</v>
@@ -4188,7 +4200,7 @@
         <v>57</v>
       </c>
       <c r="N122" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O122" t="s">
         <v>66</v>
@@ -4211,7 +4223,7 @@
         <v>57</v>
       </c>
       <c r="N123" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O123" t="s">
         <v>66</v>
@@ -4271,7 +4283,7 @@
     </row>
     <row r="129" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -4398,7 +4410,7 @@
         <v>100</v>
       </c>
       <c r="O135" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="136" spans="1:15" x14ac:dyDescent="0.25">
@@ -4416,7 +4428,7 @@
         <v>101</v>
       </c>
       <c r="O136" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="137" spans="1:15" x14ac:dyDescent="0.25">
@@ -4436,7 +4448,7 @@
         <v>5</v>
       </c>
       <c r="N137" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="O137" t="s">
         <v>7</v>
@@ -4481,7 +4493,7 @@
         <v>45</v>
       </c>
       <c r="E140" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K140" t="s">
         <v>4</v>
@@ -4501,7 +4513,7 @@
         <v>45</v>
       </c>
       <c r="E141" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K141" t="s">
         <v>97</v>
@@ -4525,7 +4537,7 @@
         <v>45</v>
       </c>
       <c r="E142" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K142" t="s">
         <v>98</v>
@@ -4617,7 +4629,7 @@
         <v>45</v>
       </c>
       <c r="E146" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K146" t="s">
         <v>4</v>
@@ -4637,7 +4649,7 @@
         <v>45</v>
       </c>
       <c r="E147" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K147" t="s">
         <v>97</v>
@@ -4653,7 +4665,7 @@
         <v>102</v>
       </c>
       <c r="O147" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="148" spans="1:15" x14ac:dyDescent="0.25">
@@ -4661,7 +4673,7 @@
         <v>45</v>
       </c>
       <c r="E148" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K148" t="s">
         <v>98</v>
@@ -4677,7 +4689,7 @@
         <v>103</v>
       </c>
       <c r="O148" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="149" spans="1:15" x14ac:dyDescent="0.25">
@@ -4793,7 +4805,7 @@
         <v>1</v>
       </c>
       <c r="D156" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G156" s="5"/>
       <c r="K156" t="s">
@@ -4817,7 +4829,7 @@
         <v>1</v>
       </c>
       <c r="D157" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G157" s="5"/>
       <c r="K157" t="s">
@@ -4838,7 +4850,7 @@
         <v>1</v>
       </c>
       <c r="D158" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G158" s="5"/>
       <c r="K158" t="s">
@@ -4859,7 +4871,7 @@
         <v>1</v>
       </c>
       <c r="D159" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G159" s="5"/>
       <c r="K159" s="45" t="s">
@@ -4878,7 +4890,7 @@
         <v>1</v>
       </c>
       <c r="D160" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G160" s="5"/>
       <c r="K160" s="45" t="s">
@@ -4897,7 +4909,7 @@
         <v>1</v>
       </c>
       <c r="D161" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G161" s="5"/>
       <c r="K161" s="45" t="s">
@@ -4916,7 +4928,7 @@
         <v>1</v>
       </c>
       <c r="D162" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G162" s="5"/>
       <c r="K162" s="45" t="s">
@@ -4935,7 +4947,7 @@
         <v>1</v>
       </c>
       <c r="D163" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G163" s="5"/>
       <c r="K163" s="45" t="s">
@@ -4954,7 +4966,7 @@
         <v>1</v>
       </c>
       <c r="D164" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G164" s="5"/>
       <c r="K164" s="45" t="s">
@@ -4973,7 +4985,7 @@
         <v>1</v>
       </c>
       <c r="D165" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G165" s="5"/>
       <c r="K165" s="45" t="s">
@@ -4992,7 +5004,7 @@
         <v>1</v>
       </c>
       <c r="D166" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G166" s="5"/>
       <c r="K166" s="45" t="s">
@@ -5011,7 +5023,7 @@
         <v>1</v>
       </c>
       <c r="D167" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G167" s="5"/>
       <c r="K167" s="45" t="s">
@@ -5030,7 +5042,7 @@
         <v>1</v>
       </c>
       <c r="D168" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G168" s="5"/>
       <c r="K168" s="45" t="s">
@@ -5049,7 +5061,7 @@
         <v>1</v>
       </c>
       <c r="D169" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G169" s="5"/>
       <c r="K169" s="45" t="s">
@@ -5068,7 +5080,7 @@
         <v>1</v>
       </c>
       <c r="D170" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G170" s="5"/>
       <c r="K170" s="45" t="s">
@@ -5559,7 +5571,7 @@
         <v>87</v>
       </c>
       <c r="O195" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="196" spans="1:15" x14ac:dyDescent="0.25">
@@ -5580,7 +5592,7 @@
         <v>79</v>
       </c>
       <c r="O196" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="197" spans="1:15" x14ac:dyDescent="0.25">
@@ -5601,7 +5613,7 @@
         <v>80</v>
       </c>
       <c r="O197" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="198" spans="1:15" x14ac:dyDescent="0.25">
@@ -5624,7 +5636,7 @@
         <v>88</v>
       </c>
       <c r="O198" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="199" spans="1:15" x14ac:dyDescent="0.25">
@@ -5644,7 +5656,7 @@
         <v>79</v>
       </c>
       <c r="O199" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="200" spans="1:15" x14ac:dyDescent="0.25">
@@ -5664,7 +5676,7 @@
         <v>80</v>
       </c>
       <c r="O200" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="201" spans="1:15" x14ac:dyDescent="0.25">
@@ -5687,7 +5699,7 @@
         <v>89</v>
       </c>
       <c r="O201" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="202" spans="1:15" x14ac:dyDescent="0.25">
@@ -5707,7 +5719,7 @@
         <v>79</v>
       </c>
       <c r="O202" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="203" spans="1:15" x14ac:dyDescent="0.25">
@@ -5727,7 +5739,7 @@
         <v>80</v>
       </c>
       <c r="O203" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="204" spans="1:15" x14ac:dyDescent="0.25">
@@ -5751,7 +5763,7 @@
         <v>90</v>
       </c>
       <c r="O204" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="205" spans="1:15" x14ac:dyDescent="0.25">
@@ -5772,7 +5784,7 @@
         <v>79</v>
       </c>
       <c r="O205" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="206" spans="1:15" x14ac:dyDescent="0.25">
@@ -5793,7 +5805,7 @@
         <v>80</v>
       </c>
       <c r="O206" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="207" spans="1:15" x14ac:dyDescent="0.25">
@@ -5814,10 +5826,10 @@
         <v>78</v>
       </c>
       <c r="N207" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="O207" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="208" spans="1:15" x14ac:dyDescent="0.25">
@@ -5838,7 +5850,7 @@
         <v>79</v>
       </c>
       <c r="O208" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="209" spans="1:15" x14ac:dyDescent="0.25">
@@ -5859,7 +5871,7 @@
         <v>80</v>
       </c>
       <c r="O209" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="210" spans="1:15" x14ac:dyDescent="0.25">
@@ -5883,7 +5895,7 @@
         <v>91</v>
       </c>
       <c r="O210" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="211" spans="1:15" x14ac:dyDescent="0.25">
@@ -5904,7 +5916,7 @@
         <v>79</v>
       </c>
       <c r="O211" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="212" spans="1:15" x14ac:dyDescent="0.25">
@@ -5925,7 +5937,7 @@
         <v>80</v>
       </c>
       <c r="O212" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="213" spans="1:15" x14ac:dyDescent="0.25">
@@ -6034,7 +6046,7 @@
     </row>
     <row r="221" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A221" s="7" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B221" s="8"/>
       <c r="C221" s="8"/>
@@ -6056,7 +6068,7 @@
     </row>
     <row r="223" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G223" s="5"/>
     </row>
@@ -6090,7 +6102,7 @@
         <v>49</v>
       </c>
       <c r="O225" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="226" spans="1:15" x14ac:dyDescent="0.25">
@@ -6116,7 +6128,7 @@
         <v>49</v>
       </c>
       <c r="O226" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="227" spans="1:15" x14ac:dyDescent="0.25">
@@ -6142,7 +6154,7 @@
         <v>49</v>
       </c>
       <c r="O227" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="228" spans="1:15" x14ac:dyDescent="0.25">
@@ -6165,7 +6177,7 @@
         <v>49</v>
       </c>
       <c r="O228" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="229" spans="1:15" x14ac:dyDescent="0.25">
@@ -6188,7 +6200,7 @@
         <v>49</v>
       </c>
       <c r="O229" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="230" spans="1:15" x14ac:dyDescent="0.25">
@@ -6196,7 +6208,7 @@
         <v>1</v>
       </c>
       <c r="E230" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G230" t="s">
         <v>17</v>
@@ -6211,7 +6223,7 @@
         <v>49</v>
       </c>
       <c r="O230" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="231" spans="1:15" x14ac:dyDescent="0.25">
@@ -6231,7 +6243,7 @@
         <v>49</v>
       </c>
       <c r="O231" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="232" spans="1:15" x14ac:dyDescent="0.25">
@@ -6239,7 +6251,7 @@
         <v>1</v>
       </c>
       <c r="G232" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K232" t="s">
         <v>25</v>
@@ -6251,7 +6263,7 @@
         <v>49</v>
       </c>
       <c r="O232" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="233" spans="1:15" x14ac:dyDescent="0.25">
@@ -6275,7 +6287,7 @@
       </c>
       <c r="N233" s="1"/>
       <c r="O233" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="234" spans="1:15" x14ac:dyDescent="0.25">
@@ -6304,7 +6316,7 @@
       </c>
       <c r="N234" s="1"/>
       <c r="O234" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="235" spans="1:15" x14ac:dyDescent="0.25">
@@ -6333,7 +6345,7 @@
       </c>
       <c r="N235" s="1"/>
       <c r="O235" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="236" spans="1:15" x14ac:dyDescent="0.25">
@@ -6362,7 +6374,7 @@
       </c>
       <c r="N236" s="1"/>
       <c r="O236" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="237" spans="1:15" x14ac:dyDescent="0.25">
@@ -6391,7 +6403,7 @@
       </c>
       <c r="N237" s="1"/>
       <c r="O237" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="238" spans="1:15" x14ac:dyDescent="0.25">
@@ -6420,7 +6432,7 @@
       </c>
       <c r="N238" s="1"/>
       <c r="O238" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="239" spans="1:15" x14ac:dyDescent="0.25">
@@ -6449,7 +6461,7 @@
       </c>
       <c r="N239" s="1"/>
       <c r="O239" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="240" spans="1:15" x14ac:dyDescent="0.25">
@@ -6478,7 +6490,7 @@
       </c>
       <c r="N240" s="1"/>
       <c r="O240" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="241" spans="1:15" x14ac:dyDescent="0.25">
@@ -6507,7 +6519,7 @@
       </c>
       <c r="N241" s="1"/>
       <c r="O241" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="242" spans="1:15" x14ac:dyDescent="0.25">
@@ -6527,7 +6539,7 @@
         <v>49</v>
       </c>
       <c r="O242" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="243" spans="1:15" x14ac:dyDescent="0.25">
@@ -6547,7 +6559,7 @@
         <v>49</v>
       </c>
       <c r="O243" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="244" spans="1:15" x14ac:dyDescent="0.25">
@@ -6567,7 +6579,7 @@
         <v>49</v>
       </c>
       <c r="O244" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="245" spans="1:15" x14ac:dyDescent="0.25">
@@ -6575,7 +6587,7 @@
         <v>35</v>
       </c>
       <c r="G245" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K245" t="s">
         <v>25</v>
@@ -6587,7 +6599,7 @@
         <v>49</v>
       </c>
       <c r="O245" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="246" spans="1:15" x14ac:dyDescent="0.25">
@@ -6616,7 +6628,7 @@
       </c>
       <c r="N246" s="1"/>
       <c r="O246" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="247" spans="1:15" x14ac:dyDescent="0.25">
@@ -6645,7 +6657,7 @@
       </c>
       <c r="N247" s="1"/>
       <c r="O247" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="248" spans="1:15" x14ac:dyDescent="0.25">
@@ -6674,7 +6686,7 @@
       </c>
       <c r="N248" s="1"/>
       <c r="O248" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="249" spans="1:15" x14ac:dyDescent="0.25">
@@ -6697,7 +6709,7 @@
         <v>49</v>
       </c>
       <c r="O249" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="250" spans="1:15" x14ac:dyDescent="0.25">
@@ -6720,7 +6732,7 @@
         <v>49</v>
       </c>
       <c r="O250" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="251" spans="1:15" x14ac:dyDescent="0.25">
@@ -6743,7 +6755,7 @@
         <v>49</v>
       </c>
       <c r="O251" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="252" spans="1:15" x14ac:dyDescent="0.25">
@@ -6773,7 +6785,7 @@
     </row>
     <row r="255" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H255" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I255" s="6"/>
       <c r="J255" s="6"/>
@@ -6788,7 +6800,7 @@
     </row>
     <row r="256" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H256" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I256" s="6"/>
       <c r="J256" s="6"/>
@@ -6807,7 +6819,7 @@
       <c r="I257" s="6"/>
       <c r="J257" s="6"/>
       <c r="K257" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L257" s="6">
         <v>0</v>
@@ -6829,7 +6841,7 @@
         <v>16</v>
       </c>
       <c r="H259" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I259" t="s">
         <v>19</v>
@@ -6838,13 +6850,16 @@
         <v>20</v>
       </c>
       <c r="L259">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M259" t="s">
         <v>49</v>
       </c>
+      <c r="N259" t="s">
+        <v>211</v>
+      </c>
       <c r="O259" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="260" spans="1:15" x14ac:dyDescent="0.25">
@@ -6855,7 +6870,7 @@
         <v>17</v>
       </c>
       <c r="H260" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I260" t="s">
         <v>19</v>
@@ -6870,7 +6885,7 @@
         <v>49</v>
       </c>
       <c r="O260" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="261" spans="1:15" x14ac:dyDescent="0.25">
@@ -6881,7 +6896,7 @@
         <v>18</v>
       </c>
       <c r="H261" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I261" t="s">
         <v>19</v>
@@ -6890,13 +6905,13 @@
         <v>20</v>
       </c>
       <c r="L261">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="M261" t="s">
         <v>49</v>
       </c>
       <c r="O261" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="262" spans="1:15" x14ac:dyDescent="0.25">
@@ -6904,10 +6919,10 @@
         <v>1</v>
       </c>
       <c r="G262" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H262" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I262" t="s">
         <v>19</v>
@@ -6916,13 +6931,16 @@
         <v>20</v>
       </c>
       <c r="L262">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M262" t="s">
         <v>49</v>
       </c>
+      <c r="N262" t="s">
+        <v>214</v>
+      </c>
       <c r="O262" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="263" spans="1:15" x14ac:dyDescent="0.25">
@@ -6933,7 +6951,7 @@
         <v>17</v>
       </c>
       <c r="H263" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I263" t="s">
         <v>19</v>
@@ -6949,7 +6967,7 @@
       </c>
       <c r="N263" s="1"/>
       <c r="O263" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="264" spans="1:15" x14ac:dyDescent="0.25">
@@ -6960,7 +6978,7 @@
         <v>18</v>
       </c>
       <c r="H264" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I264" t="s">
         <v>19</v>
@@ -6976,7 +6994,7 @@
       </c>
       <c r="N264" s="1"/>
       <c r="O264" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="265" spans="1:15" x14ac:dyDescent="0.25">
@@ -6987,7 +7005,7 @@
         <v>166</v>
       </c>
       <c r="H265" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I265" t="s">
         <v>19</v>
@@ -7003,7 +7021,7 @@
       </c>
       <c r="N265" s="1"/>
       <c r="O265" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="266" spans="1:15" x14ac:dyDescent="0.25">
@@ -7014,7 +7032,7 @@
         <v>17</v>
       </c>
       <c r="H266" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I266" t="s">
         <v>19</v>
@@ -7023,14 +7041,14 @@
         <v>20</v>
       </c>
       <c r="L266">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="M266" t="s">
         <v>49</v>
       </c>
       <c r="N266" s="1"/>
       <c r="O266" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="267" spans="1:15" x14ac:dyDescent="0.25">
@@ -7041,7 +7059,7 @@
         <v>18</v>
       </c>
       <c r="H267" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I267" t="s">
         <v>19</v>
@@ -7050,14 +7068,14 @@
         <v>20</v>
       </c>
       <c r="L267">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="M267" t="s">
         <v>49</v>
       </c>
       <c r="N267" s="1"/>
       <c r="O267" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="268" spans="1:15" x14ac:dyDescent="0.25">
@@ -7068,7 +7086,7 @@
         <v>16</v>
       </c>
       <c r="H268" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I268" t="s">
         <v>19</v>
@@ -7077,13 +7095,13 @@
         <v>20</v>
       </c>
       <c r="L268">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M268" t="s">
         <v>49</v>
       </c>
       <c r="O268" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="269" spans="1:15" x14ac:dyDescent="0.25">
@@ -7094,7 +7112,7 @@
         <v>17</v>
       </c>
       <c r="H269" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I269" t="s">
         <v>19</v>
@@ -7103,13 +7121,13 @@
         <v>20</v>
       </c>
       <c r="L269">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M269" t="s">
         <v>49</v>
       </c>
       <c r="O269" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="270" spans="1:15" x14ac:dyDescent="0.25">
@@ -7120,7 +7138,7 @@
         <v>18</v>
       </c>
       <c r="H270" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I270" t="s">
         <v>19</v>
@@ -7129,13 +7147,16 @@
         <v>20</v>
       </c>
       <c r="L270">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="M270" t="s">
         <v>49</v>
       </c>
+      <c r="N270" t="s">
+        <v>213</v>
+      </c>
       <c r="O270" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="271" spans="1:15" x14ac:dyDescent="0.25">
@@ -7143,10 +7164,10 @@
         <v>35</v>
       </c>
       <c r="G271" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H271" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I271" t="s">
         <v>19</v>
@@ -7155,24 +7176,30 @@
         <v>20</v>
       </c>
       <c r="L271">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M271" t="s">
         <v>49</v>
       </c>
+      <c r="N271" t="s">
+        <v>214</v>
+      </c>
       <c r="O271" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="272" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>45</v>
+        <v>35</v>
+      </c>
+      <c r="E272" t="s">
+        <v>41</v>
       </c>
       <c r="G272" t="s">
         <v>16</v>
       </c>
       <c r="H272" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I272" t="s">
         <v>19</v>
@@ -7181,24 +7208,27 @@
         <v>20</v>
       </c>
       <c r="L272">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M272" t="s">
         <v>49</v>
       </c>
       <c r="O272" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="273" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>45</v>
+        <v>35</v>
+      </c>
+      <c r="E273" t="s">
+        <v>41</v>
       </c>
       <c r="G273" t="s">
         <v>17</v>
       </c>
       <c r="H273" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I273" t="s">
         <v>19</v>
@@ -7207,24 +7237,27 @@
         <v>20</v>
       </c>
       <c r="L273">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M273" t="s">
         <v>49</v>
       </c>
       <c r="O273" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="274" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>45</v>
+        <v>35</v>
+      </c>
+      <c r="E274" t="s">
+        <v>41</v>
       </c>
       <c r="G274" t="s">
         <v>18</v>
       </c>
       <c r="H274" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I274" t="s">
         <v>19</v>
@@ -7233,27 +7266,27 @@
         <v>20</v>
       </c>
       <c r="L274">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="M274" t="s">
         <v>49</v>
       </c>
       <c r="O274" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="275" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E275" t="s">
-        <v>205</v>
+        <v>41</v>
       </c>
       <c r="G275" t="s">
-        <v>18</v>
+        <v>173</v>
       </c>
       <c r="H275" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I275" t="s">
         <v>19</v>
@@ -7262,27 +7295,24 @@
         <v>20</v>
       </c>
       <c r="L275">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="M275" t="s">
         <v>49</v>
       </c>
       <c r="O275" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="276" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>45</v>
       </c>
-      <c r="E276" t="s">
-        <v>47</v>
-      </c>
       <c r="G276" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H276" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I276" t="s">
         <v>19</v>
@@ -7296,186 +7326,180 @@
       <c r="M276" t="s">
         <v>49</v>
       </c>
+      <c r="N276" t="s">
+        <v>215</v>
+      </c>
       <c r="O276" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
     </row>
     <row r="277" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A277" s="1"/>
-      <c r="B277" s="1"/>
-      <c r="C277" s="1"/>
-      <c r="D277" s="1"/>
-      <c r="E277" s="1"/>
-      <c r="F277" s="1"/>
-      <c r="G277" s="1"/>
-      <c r="H277" s="1"/>
-      <c r="I277" s="1"/>
-      <c r="J277" s="1"/>
-      <c r="K277" s="1"/>
-      <c r="L277" s="1"/>
-      <c r="M277" s="1"/>
-      <c r="N277" s="1"/>
+      <c r="A277" t="s">
+        <v>45</v>
+      </c>
+      <c r="G277" t="s">
+        <v>17</v>
+      </c>
+      <c r="H277" t="s">
+        <v>183</v>
+      </c>
+      <c r="I277" t="s">
+        <v>19</v>
+      </c>
+      <c r="K277" t="s">
+        <v>20</v>
+      </c>
+      <c r="L277">
+        <v>10</v>
+      </c>
+      <c r="M277" t="s">
+        <v>49</v>
+      </c>
+      <c r="N277" t="s">
+        <v>215</v>
+      </c>
+      <c r="O277" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="278" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="G278" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H278" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I278" t="s">
         <v>19</v>
       </c>
       <c r="K278" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L278">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="M278" t="s">
         <v>49</v>
       </c>
       <c r="O278" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
     </row>
     <row r="279" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>1</v>
-      </c>
-      <c r="C279" t="s">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="E279" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="G279" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H279" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I279" t="s">
         <v>19</v>
       </c>
       <c r="K279" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L279">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="M279" t="s">
         <v>49</v>
       </c>
       <c r="O279" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
     </row>
     <row r="280" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>1</v>
-      </c>
-      <c r="C280" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="E280" t="s">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="G280" t="s">
         <v>17</v>
       </c>
       <c r="H280" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I280" t="s">
         <v>19</v>
       </c>
       <c r="K280" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L280">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="M280" t="s">
         <v>49</v>
       </c>
       <c r="O280" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
     </row>
     <row r="281" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="E281" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="G281" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H281" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I281" t="s">
         <v>19</v>
       </c>
       <c r="K281" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L281">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="M281" t="s">
         <v>49</v>
       </c>
       <c r="O281" t="s">
-        <v>172</v>
+        <v>212</v>
       </c>
     </row>
     <row r="282" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A282" t="s">
-        <v>1</v>
-      </c>
-      <c r="E282" t="s">
-        <v>8</v>
-      </c>
-      <c r="G282" t="s">
-        <v>17</v>
-      </c>
-      <c r="H282" t="s">
-        <v>184</v>
-      </c>
-      <c r="I282" t="s">
-        <v>19</v>
-      </c>
-      <c r="K282" t="s">
-        <v>21</v>
-      </c>
-      <c r="L282">
-        <v>18</v>
-      </c>
-      <c r="M282" t="s">
-        <v>49</v>
-      </c>
-      <c r="O282" t="s">
-        <v>172</v>
-      </c>
+      <c r="A282" s="1"/>
+      <c r="B282" s="1"/>
+      <c r="C282" s="1"/>
+      <c r="D282" s="1"/>
+      <c r="E282" s="1"/>
+      <c r="F282" s="1"/>
+      <c r="G282" s="1"/>
+      <c r="H282" s="1"/>
+      <c r="I282" s="1"/>
+      <c r="J282" s="1"/>
+      <c r="K282" s="1"/>
+      <c r="L282" s="1"/>
+      <c r="M282" s="1"/>
+      <c r="N282" s="1"/>
     </row>
     <row r="283" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>1</v>
       </c>
-      <c r="E283" t="s">
-        <v>196</v>
-      </c>
       <c r="G283" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H283" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I283" t="s">
         <v>19</v>
@@ -7484,24 +7508,30 @@
         <v>21</v>
       </c>
       <c r="L283">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="M283" t="s">
         <v>49</v>
       </c>
       <c r="O283" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="284" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>1</v>
       </c>
+      <c r="C284" t="s">
+        <v>2</v>
+      </c>
+      <c r="E284" t="s">
+        <v>3</v>
+      </c>
       <c r="G284" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H284" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I284" t="s">
         <v>19</v>
@@ -7510,24 +7540,30 @@
         <v>21</v>
       </c>
       <c r="L284">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="M284" t="s">
         <v>49</v>
       </c>
       <c r="O284" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="285" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>1</v>
       </c>
+      <c r="C285" t="s">
+        <v>6</v>
+      </c>
+      <c r="E285" t="s">
+        <v>3</v>
+      </c>
       <c r="G285" t="s">
-        <v>174</v>
+        <v>17</v>
       </c>
       <c r="H285" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I285" t="s">
         <v>19</v>
@@ -7536,24 +7572,27 @@
         <v>21</v>
       </c>
       <c r="L285">
-        <v>2.75</v>
+        <v>17</v>
       </c>
       <c r="M285" t="s">
         <v>49</v>
       </c>
       <c r="O285" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="286" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>54</v>
+        <v>1</v>
+      </c>
+      <c r="E286" t="s">
+        <v>9</v>
       </c>
       <c r="G286" t="s">
         <v>17</v>
       </c>
       <c r="H286" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I286" t="s">
         <v>19</v>
@@ -7562,25 +7601,27 @@
         <v>21</v>
       </c>
       <c r="L286">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="M286" t="s">
         <v>49</v>
       </c>
-      <c r="N286" s="1"/>
       <c r="O286" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="287" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>54</v>
+        <v>1</v>
+      </c>
+      <c r="E287" t="s">
+        <v>8</v>
       </c>
       <c r="G287" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H287" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I287" t="s">
         <v>19</v>
@@ -7589,25 +7630,27 @@
         <v>21</v>
       </c>
       <c r="L287">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="M287" t="s">
         <v>49</v>
       </c>
-      <c r="N287" s="1"/>
       <c r="O287" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="288" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>54</v>
+        <v>1</v>
+      </c>
+      <c r="E288" t="s">
+        <v>195</v>
       </c>
       <c r="G288" t="s">
-        <v>166</v>
+        <v>17</v>
       </c>
       <c r="H288" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I288" t="s">
         <v>19</v>
@@ -7615,28 +7658,25 @@
       <c r="K288" t="s">
         <v>21</v>
       </c>
-      <c r="L288" s="5">
-        <v>25</v>
+      <c r="L288">
+        <v>17</v>
       </c>
       <c r="M288" t="s">
         <v>49</v>
       </c>
-      <c r="N288" s="5" t="s">
-        <v>211</v>
-      </c>
       <c r="O288" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="289" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="G289" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H289" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I289" t="s">
         <v>19</v>
@@ -7645,25 +7685,24 @@
         <v>21</v>
       </c>
       <c r="L289">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="M289" t="s">
         <v>49</v>
       </c>
-      <c r="N289" s="1"/>
       <c r="O289" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="290" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="G290" t="s">
-        <v>18</v>
+        <v>173</v>
       </c>
       <c r="H290" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I290" t="s">
         <v>19</v>
@@ -7672,25 +7711,24 @@
         <v>21</v>
       </c>
       <c r="L290">
-        <v>33</v>
+        <v>2.75</v>
       </c>
       <c r="M290" t="s">
         <v>49</v>
       </c>
-      <c r="N290" s="1"/>
       <c r="O290" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="291" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G291" t="s">
-        <v>166</v>
+        <v>17</v>
       </c>
       <c r="H291" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I291" t="s">
         <v>19</v>
@@ -7698,28 +7736,26 @@
       <c r="K291" t="s">
         <v>21</v>
       </c>
-      <c r="L291" s="5">
+      <c r="L291">
         <v>25</v>
       </c>
       <c r="M291" t="s">
         <v>49</v>
       </c>
-      <c r="N291" s="5" t="s">
-        <v>211</v>
-      </c>
+      <c r="N291" s="1"/>
       <c r="O291" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="292" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="G292" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H292" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I292" t="s">
         <v>19</v>
@@ -7728,24 +7764,25 @@
         <v>21</v>
       </c>
       <c r="L292">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="M292" t="s">
         <v>49</v>
       </c>
+      <c r="N292" s="1"/>
       <c r="O292" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="293" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="G293" t="s">
-        <v>17</v>
+        <v>166</v>
       </c>
       <c r="H293" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I293" t="s">
         <v>19</v>
@@ -7753,25 +7790,28 @@
       <c r="K293" t="s">
         <v>21</v>
       </c>
-      <c r="L293">
-        <v>18</v>
+      <c r="L293" s="5">
+        <v>25</v>
       </c>
       <c r="M293" t="s">
         <v>49</v>
       </c>
+      <c r="N293" s="5" t="s">
+        <v>210</v>
+      </c>
       <c r="O293" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="294" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="G294" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H294" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I294" t="s">
         <v>19</v>
@@ -7780,24 +7820,25 @@
         <v>21</v>
       </c>
       <c r="L294">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="M294" t="s">
         <v>49</v>
       </c>
+      <c r="N294" s="1"/>
       <c r="O294" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="295" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="G295" t="s">
-        <v>174</v>
+        <v>18</v>
       </c>
       <c r="H295" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I295" t="s">
         <v>19</v>
@@ -7806,24 +7847,25 @@
         <v>21</v>
       </c>
       <c r="L295">
-        <v>2.75</v>
+        <v>33</v>
       </c>
       <c r="M295" t="s">
         <v>49</v>
       </c>
+      <c r="N295" s="1"/>
       <c r="O295" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="296" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G296" t="s">
-        <v>16</v>
+        <v>166</v>
       </c>
       <c r="H296" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I296" t="s">
         <v>19</v>
@@ -7831,25 +7873,28 @@
       <c r="K296" t="s">
         <v>21</v>
       </c>
-      <c r="L296">
-        <v>4</v>
+      <c r="L296" s="5">
+        <v>25</v>
       </c>
       <c r="M296" t="s">
         <v>49</v>
       </c>
+      <c r="N296" s="5" t="s">
+        <v>210</v>
+      </c>
       <c r="O296" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="297" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G297" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H297" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I297" t="s">
         <v>19</v>
@@ -7858,24 +7903,24 @@
         <v>21</v>
       </c>
       <c r="L297">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="M297" t="s">
         <v>49</v>
       </c>
       <c r="O297" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="298" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G298" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H298" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I298" t="s">
         <v>19</v>
@@ -7884,27 +7929,24 @@
         <v>21</v>
       </c>
       <c r="L298">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M298" t="s">
         <v>49</v>
       </c>
       <c r="O298" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="299" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>45</v>
-      </c>
-      <c r="E299" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G299" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H299" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I299" t="s">
         <v>19</v>
@@ -7913,27 +7955,24 @@
         <v>21</v>
       </c>
       <c r="L299">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="M299" t="s">
         <v>49</v>
       </c>
       <c r="O299" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="300" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>45</v>
-      </c>
-      <c r="E300" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G300" t="s">
-        <v>18</v>
+        <v>173</v>
       </c>
       <c r="H300" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I300" t="s">
         <v>19</v>
@@ -7942,105 +7981,149 @@
         <v>21</v>
       </c>
       <c r="L300">
-        <v>5</v>
+        <v>2.75</v>
       </c>
       <c r="M300" t="s">
         <v>49</v>
       </c>
       <c r="O300" t="s">
-        <v>172</v>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="301" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>45</v>
+      </c>
+      <c r="G301" t="s">
+        <v>16</v>
+      </c>
+      <c r="H301" t="s">
+        <v>183</v>
+      </c>
+      <c r="I301" t="s">
+        <v>19</v>
+      </c>
+      <c r="K301" t="s">
+        <v>21</v>
+      </c>
+      <c r="L301">
+        <v>4</v>
+      </c>
+      <c r="M301" t="s">
+        <v>49</v>
+      </c>
+      <c r="O301" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="302" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
+        <v>45</v>
+      </c>
       <c r="G302" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H302" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I302" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K302" t="s">
-        <v>192</v>
+        <v>21</v>
       </c>
       <c r="L302">
-        <v>0.01</v>
+        <v>12</v>
       </c>
       <c r="M302" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O302" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="303" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
+        <v>45</v>
+      </c>
       <c r="G303" t="s">
+        <v>18</v>
+      </c>
+      <c r="H303" t="s">
+        <v>183</v>
+      </c>
+      <c r="I303" t="s">
+        <v>19</v>
+      </c>
+      <c r="K303" t="s">
+        <v>21</v>
+      </c>
+      <c r="L303">
+        <v>20</v>
+      </c>
+      <c r="M303" t="s">
+        <v>49</v>
+      </c>
+      <c r="O303" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="304" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
+        <v>45</v>
+      </c>
+      <c r="E304" t="s">
+        <v>47</v>
+      </c>
+      <c r="G304" t="s">
         <v>17</v>
       </c>
-      <c r="H303" t="s">
-        <v>184</v>
-      </c>
-      <c r="I303" t="s">
-        <v>22</v>
-      </c>
-      <c r="K303" t="s">
-        <v>192</v>
-      </c>
-      <c r="L303">
-        <v>1</v>
-      </c>
-      <c r="M303" t="s">
-        <v>50</v>
-      </c>
-      <c r="O303" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="304" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G304" t="s">
+      <c r="H304" t="s">
+        <v>183</v>
+      </c>
+      <c r="I304" t="s">
+        <v>19</v>
+      </c>
+      <c r="K304" t="s">
+        <v>21</v>
+      </c>
+      <c r="L304">
+        <v>5</v>
+      </c>
+      <c r="M304" t="s">
+        <v>49</v>
+      </c>
+      <c r="O304" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>45</v>
+      </c>
+      <c r="E305" t="s">
+        <v>47</v>
+      </c>
+      <c r="G305" t="s">
         <v>18</v>
       </c>
-      <c r="H304" t="s">
-        <v>184</v>
-      </c>
-      <c r="I304" t="s">
-        <v>22</v>
-      </c>
-      <c r="K304" t="s">
-        <v>192</v>
-      </c>
-      <c r="L304">
-        <v>1</v>
-      </c>
-      <c r="M304" t="s">
-        <v>50</v>
-      </c>
-      <c r="O304" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G305" t="s">
-        <v>166</v>
-      </c>
       <c r="H305" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I305" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="K305" t="s">
-        <v>192</v>
+        <v>21</v>
       </c>
       <c r="L305">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M305" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O305" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="307" spans="1:15" x14ac:dyDescent="0.25">
@@ -8048,19 +8131,19 @@
         <v>16</v>
       </c>
       <c r="H307" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I307" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K307" t="s">
-        <v>21</v>
+        <v>191</v>
       </c>
       <c r="L307">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="M307" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O307" t="s">
         <v>178</v>
@@ -8071,19 +8154,19 @@
         <v>17</v>
       </c>
       <c r="H308" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I308" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K308" t="s">
-        <v>21</v>
+        <v>191</v>
       </c>
       <c r="L308">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="M308" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O308" t="s">
         <v>178</v>
@@ -8094,19 +8177,19 @@
         <v>18</v>
       </c>
       <c r="H309" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I309" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K309" t="s">
-        <v>21</v>
+        <v>191</v>
       </c>
       <c r="L309">
         <v>1</v>
       </c>
       <c r="M309" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O309" t="s">
         <v>178</v>
@@ -8114,126 +8197,117 @@
     </row>
     <row r="310" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G310" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="H310" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I310" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K310" t="s">
-        <v>21</v>
+        <v>191</v>
       </c>
       <c r="L310">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M310" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O310" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="311" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G311" t="s">
-        <v>166</v>
-      </c>
-      <c r="H311" t="s">
-        <v>184</v>
-      </c>
-      <c r="I311" t="s">
+    <row r="312" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G312" t="s">
+        <v>16</v>
+      </c>
+      <c r="H312" t="s">
+        <v>183</v>
+      </c>
+      <c r="I312" t="s">
         <v>23</v>
       </c>
-      <c r="K311" t="s">
+      <c r="K312" t="s">
         <v>21</v>
       </c>
-      <c r="L311">
-        <v>1</v>
-      </c>
-      <c r="M311" t="s">
+      <c r="L312">
+        <v>0.5</v>
+      </c>
+      <c r="M312" t="s">
         <v>49</v>
       </c>
-      <c r="O311" t="s">
-        <v>178</v>
+      <c r="O312" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="313" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G313" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H313" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I313" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K313" t="s">
-        <v>192</v>
+        <v>21</v>
       </c>
       <c r="L313">
-        <v>0.31</v>
+        <v>0.5</v>
       </c>
       <c r="M313" t="s">
-        <v>50</v>
-      </c>
-      <c r="N313" t="s">
+        <v>49</v>
+      </c>
+      <c r="O313" t="s">
         <v>177</v>
-      </c>
-      <c r="O313" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="314" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G314" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H314" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I314" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K314" t="s">
-        <v>192</v>
+        <v>21</v>
       </c>
       <c r="L314">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="M314" t="s">
-        <v>50</v>
-      </c>
-      <c r="N314" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="O314" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="315" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G315" t="s">
-        <v>18</v>
+        <v>173</v>
       </c>
       <c r="H315" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I315" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K315" t="s">
-        <v>192</v>
+        <v>21</v>
       </c>
       <c r="L315">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="M315" t="s">
-        <v>50</v>
-      </c>
-      <c r="N315" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="O315" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="316" spans="1:15" x14ac:dyDescent="0.25">
@@ -8241,85 +8315,186 @@
         <v>166</v>
       </c>
       <c r="H316" t="s">
+        <v>183</v>
+      </c>
+      <c r="I316" t="s">
+        <v>23</v>
+      </c>
+      <c r="K316" t="s">
+        <v>21</v>
+      </c>
+      <c r="L316">
+        <v>1</v>
+      </c>
+      <c r="M316" t="s">
+        <v>49</v>
+      </c>
+      <c r="O316" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="318" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G318" t="s">
+        <v>16</v>
+      </c>
+      <c r="H318" t="s">
+        <v>183</v>
+      </c>
+      <c r="I318" t="s">
+        <v>24</v>
+      </c>
+      <c r="K318" t="s">
+        <v>191</v>
+      </c>
+      <c r="L318">
+        <v>0.31</v>
+      </c>
+      <c r="M318" t="s">
+        <v>50</v>
+      </c>
+      <c r="N318" t="s">
+        <v>176</v>
+      </c>
+      <c r="O318" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="319" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G319" t="s">
+        <v>17</v>
+      </c>
+      <c r="H319" t="s">
+        <v>183</v>
+      </c>
+      <c r="I319" t="s">
+        <v>24</v>
+      </c>
+      <c r="K319" t="s">
+        <v>191</v>
+      </c>
+      <c r="L319">
+        <v>31</v>
+      </c>
+      <c r="M319" t="s">
+        <v>50</v>
+      </c>
+      <c r="N319" t="s">
+        <v>17</v>
+      </c>
+      <c r="O319" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="320" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G320" t="s">
+        <v>18</v>
+      </c>
+      <c r="H320" t="s">
+        <v>183</v>
+      </c>
+      <c r="I320" t="s">
+        <v>24</v>
+      </c>
+      <c r="K320" t="s">
+        <v>191</v>
+      </c>
+      <c r="L320">
+        <v>31</v>
+      </c>
+      <c r="M320" t="s">
+        <v>50</v>
+      </c>
+      <c r="N320" t="s">
+        <v>17</v>
+      </c>
+      <c r="O320" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="321" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G321" t="s">
+        <v>166</v>
+      </c>
+      <c r="H321" t="s">
+        <v>183</v>
+      </c>
+      <c r="I321" t="s">
+        <v>24</v>
+      </c>
+      <c r="K321" t="s">
+        <v>191</v>
+      </c>
+      <c r="L321">
+        <v>31</v>
+      </c>
+      <c r="M321" t="s">
+        <v>50</v>
+      </c>
+      <c r="N321" t="s">
+        <v>17</v>
+      </c>
+      <c r="O321" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="323" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A323" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="324" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H324" t="s">
         <v>184</v>
       </c>
-      <c r="I316" t="s">
-        <v>24</v>
-      </c>
-      <c r="K316" t="s">
-        <v>192</v>
-      </c>
-      <c r="L316">
-        <v>31</v>
-      </c>
-      <c r="M316" t="s">
-        <v>50</v>
-      </c>
-      <c r="N316" t="s">
-        <v>17</v>
-      </c>
-      <c r="O316" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="318" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A318" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="319" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="H319" t="s">
+      <c r="I324" t="s">
+        <v>184</v>
+      </c>
+      <c r="K324" t="s">
+        <v>20</v>
+      </c>
+      <c r="L324">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H325" t="s">
+        <v>184</v>
+      </c>
+      <c r="I325" t="s">
+        <v>184</v>
+      </c>
+      <c r="K325" t="s">
+        <v>21</v>
+      </c>
+      <c r="L325">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H326" t="s">
         <v>185</v>
       </c>
-      <c r="I319" t="s">
+      <c r="I326" t="s">
         <v>185</v>
       </c>
-      <c r="K319" t="s">
+      <c r="K326" t="s">
         <v>20</v>
       </c>
-      <c r="L319">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="320" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="H320" t="s">
+      <c r="L326" s="37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H327" t="s">
         <v>185</v>
       </c>
-      <c r="I320" t="s">
+      <c r="I327" t="s">
         <v>185</v>
       </c>
-      <c r="K320" t="s">
+      <c r="K327" t="s">
         <v>21</v>
       </c>
-      <c r="L320">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="321" spans="8:12" x14ac:dyDescent="0.25">
-      <c r="H321" t="s">
-        <v>186</v>
-      </c>
-      <c r="I321" t="s">
-        <v>186</v>
-      </c>
-      <c r="K321" t="s">
-        <v>20</v>
-      </c>
-      <c r="L321" s="37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="322" spans="8:12" x14ac:dyDescent="0.25">
-      <c r="H322" t="s">
-        <v>186</v>
-      </c>
-      <c r="I322" t="s">
-        <v>186</v>
-      </c>
-      <c r="K322" t="s">
-        <v>21</v>
-      </c>
-      <c r="L322">
+      <c r="L327">
         <v>0</v>
       </c>
     </row>
@@ -8471,7 +8646,7 @@
     </row>
     <row r="7" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B7" s="38" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C7" s="39" t="s">
         <v>3</v>
@@ -8483,7 +8658,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="39" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G7" s="39" t="s">
         <v>9</v>
@@ -8492,14 +8667,14 @@
       <c r="I7" s="39"/>
       <c r="J7" s="39"/>
       <c r="K7" s="39" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="L7" s="39"/>
       <c r="M7" s="39" t="s">
         <v>47</v>
       </c>
       <c r="O7" s="38" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P7" s="39" t="str">
         <f>C7</f>
@@ -8579,7 +8754,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="38" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="P8" s="41" t="str">
         <f>P5&amp;P6&amp;P7</f>
@@ -8916,7 +9091,7 @@
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B12" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C12" s="37">
         <f>C83+C97</f>
@@ -8959,7 +9134,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="39" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="P12" s="37">
         <f t="shared" si="3"/>
@@ -9311,20 +9486,20 @@
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" s="52" t="s">
+      <c r="B19" s="47" t="s">
         <v>142</v>
       </c>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
-      <c r="E19" s="52"/>
-      <c r="F19" s="52"/>
-      <c r="G19" s="52"/>
-      <c r="H19" s="52"/>
-      <c r="I19" s="52"/>
-      <c r="J19" s="52"/>
-      <c r="K19" s="52"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="52"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="47"/>
+      <c r="L19" s="47"/>
+      <c r="M19" s="47"/>
     </row>
     <row r="20" spans="2:13" ht="33" x14ac:dyDescent="0.25">
       <c r="B20" s="21" t="s">
@@ -10149,23 +10324,23 @@
       <c r="M43" s="20"/>
     </row>
     <row r="45" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B45" s="52" t="s">
+      <c r="B45" s="47" t="s">
         <v>157</v>
       </c>
-      <c r="C45" s="52"/>
-      <c r="D45" s="52"/>
-      <c r="E45" s="52"/>
-      <c r="F45" s="52"/>
-      <c r="G45" s="52"/>
-      <c r="H45" s="52"/>
-      <c r="I45" s="52"/>
-      <c r="J45" s="52"/>
-      <c r="K45" s="52"/>
-      <c r="L45" s="52"/>
-      <c r="M45" s="52"/>
-      <c r="N45" s="52"/>
-      <c r="O45" s="52"/>
-      <c r="P45" s="52"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="47"/>
+      <c r="E45" s="47"/>
+      <c r="F45" s="47"/>
+      <c r="G45" s="47"/>
+      <c r="H45" s="47"/>
+      <c r="I45" s="47"/>
+      <c r="J45" s="47"/>
+      <c r="K45" s="47"/>
+      <c r="L45" s="47"/>
+      <c r="M45" s="47"/>
+      <c r="N45" s="47"/>
+      <c r="O45" s="47"/>
+      <c r="P45" s="47"/>
     </row>
     <row r="46" spans="2:16" ht="44.25" x14ac:dyDescent="0.25">
       <c r="B46" s="31" t="s">
@@ -11133,43 +11308,43 @@
       <c r="N69" s="20"/>
     </row>
     <row r="71" spans="2:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="52" t="s">
+      <c r="B71" s="47" t="s">
         <v>150</v>
       </c>
-      <c r="C71" s="52"/>
-      <c r="D71" s="52"/>
-      <c r="E71" s="52"/>
-      <c r="F71" s="52"/>
-      <c r="G71" s="52"/>
-      <c r="H71" s="52"/>
-      <c r="I71" s="52"/>
-      <c r="J71" s="52"/>
-      <c r="K71" s="52"/>
-      <c r="L71" s="52"/>
-      <c r="M71" s="52"/>
+      <c r="C71" s="47"/>
+      <c r="D71" s="47"/>
+      <c r="E71" s="47"/>
+      <c r="F71" s="47"/>
+      <c r="G71" s="47"/>
+      <c r="H71" s="47"/>
+      <c r="I71" s="47"/>
+      <c r="J71" s="47"/>
+      <c r="K71" s="47"/>
+      <c r="L71" s="47"/>
+      <c r="M71" s="47"/>
     </row>
     <row r="72" spans="2:14" ht="24" x14ac:dyDescent="0.25">
-      <c r="B72" s="54" t="s">
+      <c r="B72" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="C72" s="56" t="s">
+      <c r="C72" s="50" t="s">
         <v>151</v>
       </c>
-      <c r="D72" s="57"/>
-      <c r="E72" s="57"/>
-      <c r="F72" s="57"/>
-      <c r="G72" s="57"/>
-      <c r="H72" s="57"/>
-      <c r="I72" s="57"/>
-      <c r="J72" s="57"/>
-      <c r="K72" s="58"/>
+      <c r="D72" s="51"/>
+      <c r="E72" s="51"/>
+      <c r="F72" s="51"/>
+      <c r="G72" s="51"/>
+      <c r="H72" s="51"/>
+      <c r="I72" s="51"/>
+      <c r="J72" s="51"/>
+      <c r="K72" s="52"/>
       <c r="L72" s="26" t="s">
         <v>152</v>
       </c>
       <c r="M72" s="27"/>
     </row>
     <row r="73" spans="2:14" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="B73" s="55"/>
+      <c r="B73" s="49"/>
       <c r="C73" s="16" t="s">
         <v>132</v>
       </c>
@@ -11588,22 +11763,22 @@
       <c r="L85" s="53"/>
     </row>
     <row r="86" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B86" s="47"/>
-      <c r="C86" s="49" t="s">
+      <c r="B86" s="54"/>
+      <c r="C86" s="56" t="s">
         <v>155</v>
       </c>
-      <c r="D86" s="50"/>
-      <c r="E86" s="50"/>
-      <c r="F86" s="50"/>
-      <c r="G86" s="50"/>
-      <c r="H86" s="50"/>
-      <c r="I86" s="50"/>
-      <c r="J86" s="50"/>
-      <c r="K86" s="51"/>
+      <c r="D86" s="57"/>
+      <c r="E86" s="57"/>
+      <c r="F86" s="57"/>
+      <c r="G86" s="57"/>
+      <c r="H86" s="57"/>
+      <c r="I86" s="57"/>
+      <c r="J86" s="57"/>
+      <c r="K86" s="58"/>
       <c r="L86" s="20"/>
     </row>
     <row r="87" spans="2:13" ht="42" x14ac:dyDescent="0.25">
-      <c r="B87" s="48"/>
+      <c r="B87" s="55"/>
       <c r="C87" s="29" t="s">
         <v>132</v>
       </c>
@@ -11973,16 +12148,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B86:B87"/>
+    <mergeCell ref="C86:K86"/>
+    <mergeCell ref="B45:P45"/>
+    <mergeCell ref="B58:N58"/>
+    <mergeCell ref="B32:M32"/>
     <mergeCell ref="B19:M19"/>
     <mergeCell ref="B71:M71"/>
     <mergeCell ref="B72:B73"/>
     <mergeCell ref="C72:K72"/>
     <mergeCell ref="B85:L85"/>
-    <mergeCell ref="B86:B87"/>
-    <mergeCell ref="C86:K86"/>
-    <mergeCell ref="B45:P45"/>
-    <mergeCell ref="B58:N58"/>
-    <mergeCell ref="B32:M32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added NOx and N2 losses for MMS='anaerobic digestion'
</commit_message>
<xml_diff>
--- a/data/default/ManureMgmt.xlsx
+++ b/data/default/ManureMgmt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CCE5617-CD6F-4CE5-9E2A-5E848FF4E913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC0BD568-61C6-40F1-9963-75B76F55BF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1717" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1730" uniqueCount="216">
   <si>
     <t>value</t>
   </si>
@@ -1444,8 +1444,26 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1461,24 +1479,6 @@
     </xf>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="9"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="10"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1827,7 +1827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O327"/>
+  <dimension ref="A1:O329"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -8197,7 +8197,7 @@
     </row>
     <row r="310" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G310" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="H310" t="s">
         <v>183</v>
@@ -8209,7 +8209,7 @@
         <v>191</v>
       </c>
       <c r="L310">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="M310" t="s">
         <v>50</v>
@@ -8218,32 +8218,32 @@
         <v>178</v>
       </c>
     </row>
-    <row r="312" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G312" t="s">
-        <v>16</v>
-      </c>
-      <c r="H312" t="s">
+    <row r="311" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G311" t="s">
+        <v>166</v>
+      </c>
+      <c r="H311" t="s">
         <v>183</v>
       </c>
-      <c r="I312" t="s">
-        <v>23</v>
-      </c>
-      <c r="K312" t="s">
-        <v>21</v>
-      </c>
-      <c r="L312">
-        <v>0.5</v>
-      </c>
-      <c r="M312" t="s">
-        <v>49</v>
-      </c>
-      <c r="O312" t="s">
-        <v>177</v>
+      <c r="I311" t="s">
+        <v>22</v>
+      </c>
+      <c r="K311" t="s">
+        <v>191</v>
+      </c>
+      <c r="L311">
+        <v>1</v>
+      </c>
+      <c r="M311" t="s">
+        <v>50</v>
+      </c>
+      <c r="O311" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="313" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G313" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H313" t="s">
         <v>183</v>
@@ -8266,7 +8266,7 @@
     </row>
     <row r="314" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G314" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H314" t="s">
         <v>183</v>
@@ -8278,7 +8278,7 @@
         <v>21</v>
       </c>
       <c r="L314">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M314" t="s">
         <v>49</v>
@@ -8289,7 +8289,7 @@
     </row>
     <row r="315" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G315" t="s">
-        <v>173</v>
+        <v>18</v>
       </c>
       <c r="H315" t="s">
         <v>183</v>
@@ -8301,7 +8301,7 @@
         <v>21</v>
       </c>
       <c r="L315">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M315" t="s">
         <v>49</v>
@@ -8312,7 +8312,7 @@
     </row>
     <row r="316" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G316" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="H316" t="s">
         <v>183</v>
@@ -8324,7 +8324,7 @@
         <v>21</v>
       </c>
       <c r="L316">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M316" t="s">
         <v>49</v>
@@ -8333,35 +8333,32 @@
         <v>177</v>
       </c>
     </row>
-    <row r="318" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G318" t="s">
-        <v>16</v>
-      </c>
-      <c r="H318" t="s">
+    <row r="317" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G317" t="s">
+        <v>166</v>
+      </c>
+      <c r="H317" t="s">
         <v>183</v>
       </c>
-      <c r="I318" t="s">
-        <v>24</v>
-      </c>
-      <c r="K318" t="s">
-        <v>191</v>
-      </c>
-      <c r="L318">
-        <v>0.31</v>
-      </c>
-      <c r="M318" t="s">
-        <v>50</v>
-      </c>
-      <c r="N318" t="s">
-        <v>176</v>
-      </c>
-      <c r="O318" t="s">
-        <v>175</v>
+      <c r="I317" t="s">
+        <v>23</v>
+      </c>
+      <c r="K317" t="s">
+        <v>21</v>
+      </c>
+      <c r="L317">
+        <v>1</v>
+      </c>
+      <c r="M317" t="s">
+        <v>49</v>
+      </c>
+      <c r="O317" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="319" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G319" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H319" t="s">
         <v>183</v>
@@ -8373,13 +8370,13 @@
         <v>191</v>
       </c>
       <c r="L319">
-        <v>31</v>
+        <v>0.3</v>
       </c>
       <c r="M319" t="s">
         <v>50</v>
       </c>
       <c r="N319" t="s">
-        <v>17</v>
+        <v>176</v>
       </c>
       <c r="O319" t="s">
         <v>175</v>
@@ -8387,7 +8384,7 @@
     </row>
     <row r="320" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G320" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H320" t="s">
         <v>183</v>
@@ -8399,7 +8396,7 @@
         <v>191</v>
       </c>
       <c r="L320">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M320" t="s">
         <v>50</v>
@@ -8413,7 +8410,7 @@
     </row>
     <row r="321" spans="1:15" x14ac:dyDescent="0.25">
       <c r="G321" t="s">
-        <v>166</v>
+        <v>18</v>
       </c>
       <c r="H321" t="s">
         <v>183</v>
@@ -8425,7 +8422,7 @@
         <v>191</v>
       </c>
       <c r="L321">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M321" t="s">
         <v>50</v>
@@ -8437,64 +8434,116 @@
         <v>175</v>
       </c>
     </row>
+    <row r="322" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="G322" t="s">
+        <v>173</v>
+      </c>
+      <c r="H322" t="s">
+        <v>183</v>
+      </c>
+      <c r="I322" t="s">
+        <v>24</v>
+      </c>
+      <c r="K322" t="s">
+        <v>191</v>
+      </c>
+      <c r="L322">
+        <v>0.3</v>
+      </c>
+      <c r="M322" t="s">
+        <v>50</v>
+      </c>
+      <c r="N322" t="s">
+        <v>176</v>
+      </c>
+      <c r="O322" t="s">
+        <v>175</v>
+      </c>
+    </row>
     <row r="323" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A323" s="1" t="s">
+      <c r="G323" t="s">
+        <v>166</v>
+      </c>
+      <c r="H323" t="s">
+        <v>183</v>
+      </c>
+      <c r="I323" t="s">
+        <v>24</v>
+      </c>
+      <c r="K323" t="s">
+        <v>191</v>
+      </c>
+      <c r="L323">
+        <v>30</v>
+      </c>
+      <c r="M323" t="s">
+        <v>50</v>
+      </c>
+      <c r="N323" t="s">
+        <v>17</v>
+      </c>
+      <c r="O323" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="325" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A325" s="1" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="324" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="H324" t="s">
-        <v>184</v>
-      </c>
-      <c r="I324" t="s">
-        <v>184</v>
-      </c>
-      <c r="K324" t="s">
-        <v>20</v>
-      </c>
-      <c r="L324">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="325" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="H325" t="s">
-        <v>184</v>
-      </c>
-      <c r="I325" t="s">
-        <v>184</v>
-      </c>
-      <c r="K325" t="s">
-        <v>21</v>
-      </c>
-      <c r="L325">
-        <v>0</v>
       </c>
     </row>
     <row r="326" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H326" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I326" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K326" t="s">
         <v>20</v>
       </c>
-      <c r="L326" s="37">
+      <c r="L326">
         <v>0</v>
       </c>
     </row>
     <row r="327" spans="1:15" x14ac:dyDescent="0.25">
       <c r="H327" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="I327" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K327" t="s">
         <v>21</v>
       </c>
       <c r="L327">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H328" t="s">
+        <v>185</v>
+      </c>
+      <c r="I328" t="s">
+        <v>185</v>
+      </c>
+      <c r="K328" t="s">
+        <v>20</v>
+      </c>
+      <c r="L328" s="37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="H329" t="s">
+        <v>185</v>
+      </c>
+      <c r="I329" t="s">
+        <v>185</v>
+      </c>
+      <c r="K329" t="s">
+        <v>21</v>
+      </c>
+      <c r="L329">
         <v>0</v>
       </c>
     </row>
@@ -9486,20 +9535,20 @@
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="52" t="s">
         <v>142</v>
       </c>
-      <c r="C19" s="47"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="47"/>
-      <c r="I19" s="47"/>
-      <c r="J19" s="47"/>
-      <c r="K19" s="47"/>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="52"/>
+      <c r="J19" s="52"/>
+      <c r="K19" s="52"/>
+      <c r="L19" s="52"/>
+      <c r="M19" s="52"/>
     </row>
     <row r="20" spans="2:13" ht="33" x14ac:dyDescent="0.25">
       <c r="B20" s="21" t="s">
@@ -10324,23 +10373,23 @@
       <c r="M43" s="20"/>
     </row>
     <row r="45" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B45" s="47" t="s">
+      <c r="B45" s="52" t="s">
         <v>157</v>
       </c>
-      <c r="C45" s="47"/>
-      <c r="D45" s="47"/>
-      <c r="E45" s="47"/>
-      <c r="F45" s="47"/>
-      <c r="G45" s="47"/>
-      <c r="H45" s="47"/>
-      <c r="I45" s="47"/>
-      <c r="J45" s="47"/>
-      <c r="K45" s="47"/>
-      <c r="L45" s="47"/>
-      <c r="M45" s="47"/>
-      <c r="N45" s="47"/>
-      <c r="O45" s="47"/>
-      <c r="P45" s="47"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="52"/>
+      <c r="E45" s="52"/>
+      <c r="F45" s="52"/>
+      <c r="G45" s="52"/>
+      <c r="H45" s="52"/>
+      <c r="I45" s="52"/>
+      <c r="J45" s="52"/>
+      <c r="K45" s="52"/>
+      <c r="L45" s="52"/>
+      <c r="M45" s="52"/>
+      <c r="N45" s="52"/>
+      <c r="O45" s="52"/>
+      <c r="P45" s="52"/>
     </row>
     <row r="46" spans="2:16" ht="44.25" x14ac:dyDescent="0.25">
       <c r="B46" s="31" t="s">
@@ -11308,43 +11357,43 @@
       <c r="N69" s="20"/>
     </row>
     <row r="71" spans="2:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="47" t="s">
+      <c r="B71" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="C71" s="47"/>
-      <c r="D71" s="47"/>
-      <c r="E71" s="47"/>
-      <c r="F71" s="47"/>
-      <c r="G71" s="47"/>
-      <c r="H71" s="47"/>
-      <c r="I71" s="47"/>
-      <c r="J71" s="47"/>
-      <c r="K71" s="47"/>
-      <c r="L71" s="47"/>
-      <c r="M71" s="47"/>
+      <c r="C71" s="52"/>
+      <c r="D71" s="52"/>
+      <c r="E71" s="52"/>
+      <c r="F71" s="52"/>
+      <c r="G71" s="52"/>
+      <c r="H71" s="52"/>
+      <c r="I71" s="52"/>
+      <c r="J71" s="52"/>
+      <c r="K71" s="52"/>
+      <c r="L71" s="52"/>
+      <c r="M71" s="52"/>
     </row>
     <row r="72" spans="2:14" ht="24" x14ac:dyDescent="0.25">
-      <c r="B72" s="48" t="s">
+      <c r="B72" s="54" t="s">
         <v>131</v>
       </c>
-      <c r="C72" s="50" t="s">
+      <c r="C72" s="56" t="s">
         <v>151</v>
       </c>
-      <c r="D72" s="51"/>
-      <c r="E72" s="51"/>
-      <c r="F72" s="51"/>
-      <c r="G72" s="51"/>
-      <c r="H72" s="51"/>
-      <c r="I72" s="51"/>
-      <c r="J72" s="51"/>
-      <c r="K72" s="52"/>
+      <c r="D72" s="57"/>
+      <c r="E72" s="57"/>
+      <c r="F72" s="57"/>
+      <c r="G72" s="57"/>
+      <c r="H72" s="57"/>
+      <c r="I72" s="57"/>
+      <c r="J72" s="57"/>
+      <c r="K72" s="58"/>
       <c r="L72" s="26" t="s">
         <v>152</v>
       </c>
       <c r="M72" s="27"/>
     </row>
     <row r="73" spans="2:14" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="B73" s="49"/>
+      <c r="B73" s="55"/>
       <c r="C73" s="16" t="s">
         <v>132</v>
       </c>
@@ -11763,22 +11812,22 @@
       <c r="L85" s="53"/>
     </row>
     <row r="86" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B86" s="54"/>
-      <c r="C86" s="56" t="s">
+      <c r="B86" s="47"/>
+      <c r="C86" s="49" t="s">
         <v>155</v>
       </c>
-      <c r="D86" s="57"/>
-      <c r="E86" s="57"/>
-      <c r="F86" s="57"/>
-      <c r="G86" s="57"/>
-      <c r="H86" s="57"/>
-      <c r="I86" s="57"/>
-      <c r="J86" s="57"/>
-      <c r="K86" s="58"/>
+      <c r="D86" s="50"/>
+      <c r="E86" s="50"/>
+      <c r="F86" s="50"/>
+      <c r="G86" s="50"/>
+      <c r="H86" s="50"/>
+      <c r="I86" s="50"/>
+      <c r="J86" s="50"/>
+      <c r="K86" s="51"/>
       <c r="L86" s="20"/>
     </row>
     <row r="87" spans="2:13" ht="42" x14ac:dyDescent="0.25">
-      <c r="B87" s="55"/>
+      <c r="B87" s="48"/>
       <c r="C87" s="29" t="s">
         <v>132</v>
       </c>
@@ -12148,16 +12197,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B19:M19"/>
+    <mergeCell ref="B71:M71"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C72:K72"/>
+    <mergeCell ref="B85:L85"/>
     <mergeCell ref="B86:B87"/>
     <mergeCell ref="C86:K86"/>
     <mergeCell ref="B45:P45"/>
     <mergeCell ref="B58:N58"/>
     <mergeCell ref="B32:M32"/>
-    <mergeCell ref="B19:M19"/>
-    <mergeCell ref="B71:M71"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C72:K72"/>
-    <mergeCell ref="B85:L85"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>